<commit_message>
feat: capture and embed XLSX chart images at 1920×1080 (Full HD)
ImageGenerator.generate now accepts width/height kwargs (defaulting
to 800×600 for all existing callers). render_xlsx passes
ExcelExporter::CHART_WIDTH/CHART_HEIGHT (1920×1080) so chart PNGs
are captured at Full HD resolution and embedded at the same size.
Sheet orientation is set to landscape for a better viewing experience.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -76,7 +76,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7620000" cy="4762500"/>
+    <xdr:ext cx="18288000" cy="10287000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -114,7 +114,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7620000" cy="4762500"/>
+    <xdr:ext cx="18288000" cy="10287000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -152,7 +152,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7620000" cy="4762500"/>
+    <xdr:ext cx="18288000" cy="10287000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -190,7 +190,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7620000" cy="4762500"/>
+    <xdr:ext cx="18288000" cy="10287000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -228,7 +228,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7620000" cy="4762500"/>
+    <xdr:ext cx="18288000" cy="10287000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -1128,7 +1128,7 @@
   <sheetCalcPr fullCalcOnLoad="1"/>
   <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup/>
+  <pageSetup orientation="landscape"/>
   <headerFooter/>
   <drawing r:id="rId13"/>
 </worksheet>
@@ -1144,7 +1144,7 @@
   <sheetCalcPr fullCalcOnLoad="1"/>
   <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup/>
+  <pageSetup orientation="landscape"/>
   <headerFooter/>
   <drawing r:id="rId14"/>
 </worksheet>
@@ -1160,7 +1160,7 @@
   <sheetCalcPr fullCalcOnLoad="1"/>
   <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup/>
+  <pageSetup orientation="landscape"/>
   <headerFooter/>
   <drawing r:id="rId15"/>
 </worksheet>
@@ -1176,7 +1176,7 @@
   <sheetCalcPr fullCalcOnLoad="1"/>
   <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup/>
+  <pageSetup orientation="landscape"/>
   <headerFooter/>
   <drawing r:id="rId16"/>
 </worksheet>
@@ -1192,7 +1192,7 @@
   <sheetCalcPr fullCalcOnLoad="1"/>
   <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup/>
+  <pageSetup orientation="landscape"/>
   <headerFooter/>
   <drawing r:id="rId17"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: use device_scale_factor 2× for XLSX chart captures (4K-crisp PNGs)
ImageGenerator.generate now accepts a scale: kwarg (device_scale_factor,
default 1 — all existing callers unchanged). render_xlsx passes
ExcelExporter::CHART_SCALE = 2, so Playwright captures each chart at
3840×2160 physical pixels while the viewport remains 1920×1080.
The PNGs are still embedded at 1920×1080 display units so the sheet
layout is unchanged, but the 2× pixel density means Excel renders them
without upscaling blur on 4K/HiDPI screens.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -4,11 +4,6 @@
   <workbookPr date1904="false"/>
   <sheets>
     <sheet sheetId="1" name="Work Items" r:id="rId1"/>
-    <sheet sheetId="2" name="Aging Wip" r:id="rId2"/>
-    <sheet sheetId="3" name="Cfd Plot" r:id="rId3"/>
-    <sheet sheetId="4" name="Cycle Time Scatter" r:id="rId4"/>
-    <sheet sheetId="5" name="Forecasted Cfd Plot" r:id="rId5"/>
-    <sheet sheetId="6" name="Throughput Histogram" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -67,196 +62,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2336800" cy="2161540"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2336800" cy="2161540"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2336800" cy="2161540"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2336800" cy="2161540"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="" descr=""/>
-        <xdr:cNvPicPr>
-          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2336800" cy="2161540"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
   <sheetPr>
@@ -1116,84 +921,4 @@
   <pageSetup/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
-  <sheetData/>
-  <sheetCalcPr fullCalcOnLoad="1"/>
-  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
-  <headerFooter/>
-  <drawing r:id="rId13"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
-  <sheetData/>
-  <sheetCalcPr fullCalcOnLoad="1"/>
-  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
-  <headerFooter/>
-  <drawing r:id="rId14"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
-  <sheetData/>
-  <sheetCalcPr fullCalcOnLoad="1"/>
-  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
-  <headerFooter/>
-  <drawing r:id="rId15"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
-  <sheetData/>
-  <sheetCalcPr fullCalcOnLoad="1"/>
-  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
-  <headerFooter/>
-  <drawing r:id="rId16"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
-  <sheetData/>
-  <sheetCalcPr fullCalcOnLoad="1"/>
-  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
-  <headerFooter/>
-  <drawing r:id="rId17"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: raise on chart image failure; fix deviceScaleFactor casing
device_scale_factor: is not a valid playwright-ruby-client keyword —
the correct camelCase form is deviceScaleFactor:.

Per "dead programs tell no lies", generate_chart_images now raises
instead of swallowing errors. Callers that genuinely need graceful
degradation rescue at their own level:
- render_ppt_multi_slide delegates to generate_chart_images_or_warn
  (PPT is a last-resort fallback; text-only slides are acceptable)
- generate_images_if_needed warns and omits inline images for
  markdown/confluence (supplementary feature)
- render_xlsx lets the error propagate — broken chart capture means
  a broken export, and the caller should know immediately

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -4,6 +4,11 @@
   <workbookPr date1904="false"/>
   <sheets>
     <sheet sheetId="1" name="Work Items" r:id="rId1"/>
+    <sheet sheetId="2" name="Aging Wip" r:id="rId2"/>
+    <sheet sheetId="3" name="Cfd Plot" r:id="rId3"/>
+    <sheet sheetId="4" name="Cycle Time Scatter" r:id="rId4"/>
+    <sheet sheetId="5" name="Forecasted Cfd Plot" r:id="rId5"/>
+    <sheet sheetId="6" name="Throughput Histogram" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -62,6 +67,196 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2336800" cy="2161540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2336800" cy="2161540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2336800" cy="2161540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2336800" cy="2161540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2336800" cy="2161540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
   <sheetPr>
@@ -921,4 +1116,84 @@
   <pageSetup/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
+  <sheetData/>
+  <sheetCalcPr fullCalcOnLoad="1"/>
+  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter/>
+  <drawing r:id="rId13"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
+  <sheetData/>
+  <sheetCalcPr fullCalcOnLoad="1"/>
+  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter/>
+  <drawing r:id="rId14"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
+  <sheetData/>
+  <sheetCalcPr fullCalcOnLoad="1"/>
+  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter/>
+  <drawing r:id="rId15"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
+  <sheetData/>
+  <sheetCalcPr fullCalcOnLoad="1"/>
+  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter/>
+  <drawing r:id="rId16"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
+  <sheetData/>
+  <sheetCalcPr fullCalcOnLoad="1"/>
+  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter/>
+  <drawing r:id="rId17"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: polish XLSX chart sizing and add date columns to CSV export
- Read actual PNG dimensions so XLSX cells match each image exactly
- Rename CHART_WIDTH/HEIGHT → CAPTURE_WIDTH/HEIGHT for clarity
- Add YYYY-Week, YYYY-MM, YYYY columns to raw CSV for pivot-table use
- Add DONE_THRESHOLD_LABELS constant and threshold_index helper (shared by CTBOT chart)
- Extend verify-fresh-install to assert dashboard.csv and dashboard.xlsx exist
- Add Windows CI step to woodpecker publish pipeline
- Exclude scripts/*.ps1 from RuboCop

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -6,9 +6,10 @@
     <sheet sheetId="1" name="Work Items" r:id="rId1"/>
     <sheet sheetId="2" name="Aging Wip" r:id="rId2"/>
     <sheet sheetId="3" name="Cfd Plot" r:id="rId3"/>
-    <sheet sheetId="4" name="Cycle Time Scatter" r:id="rId4"/>
-    <sheet sheetId="5" name="Forecasted Cfd Plot" r:id="rId5"/>
-    <sheet sheetId="6" name="Throughput Histogram" r:id="rId6"/>
+    <sheet sheetId="4" name="Cycle Time Bands" r:id="rId4"/>
+    <sheet sheetId="5" name="Cycle Time Scatter" r:id="rId5"/>
+    <sheet sheetId="6" name="Forecasted Cfd Plot" r:id="rId6"/>
+    <sheet sheetId="7" name="Throughput Histogram" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -76,7 +77,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:ext cx="5038725" cy="4667250"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -85,7 +86,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -114,7 +115,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:ext cx="5038725" cy="4667250"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -123,7 +124,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -152,7 +153,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:ext cx="5038725" cy="4667250"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -161,7 +162,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -190,7 +191,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:ext cx="5038725" cy="4667250"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -199,7 +200,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -228,7 +229,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="18288000" cy="10287000"/>
+    <xdr:ext cx="5038725" cy="4667250"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="" descr=""/>
@@ -237,7 +238,45 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2336800" cy="2161540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5038725" cy="4667250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noSelect="1" noChangeAspect="1" noMove="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -262,7 +301,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="11.0" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -272,13 +311,16 @@
     <col width="14.3" min="5" max="5" bestFit="1" customWidth="1"/>
     <col width="14.3" min="6" max="6" bestFit="1" customWidth="1"/>
     <col width="15.400000000000002" min="7" max="7" bestFit="1" customWidth="1"/>
-    <col width="22.0" min="8" max="8" bestFit="1" customWidth="1"/>
-    <col width="23.1" min="9" max="9" bestFit="1" customWidth="1"/>
-    <col width="16.5" min="10" max="10" bestFit="1" customWidth="1"/>
-    <col width="17.6" min="11" max="11" bestFit="1" customWidth="1"/>
-    <col width="18.700000000000003" min="12" max="12" bestFit="1" customWidth="1"/>
-    <col width="18.700000000000003" min="13" max="13" bestFit="1" customWidth="1"/>
-    <col width="18.700000000000003" min="14" max="14" bestFit="1" customWidth="1"/>
+    <col width="13.200000000000001" min="8" max="8" bestFit="1" customWidth="1"/>
+    <col width="11.0" min="9" max="9" bestFit="1" customWidth="1"/>
+    <col width="7.700000000000001" min="10" max="10" bestFit="1" customWidth="1"/>
+    <col width="22.0" min="11" max="11" bestFit="1" customWidth="1"/>
+    <col width="23.1" min="12" max="12" bestFit="1" customWidth="1"/>
+    <col width="16.5" min="13" max="13" bestFit="1" customWidth="1"/>
+    <col width="17.6" min="14" max="14" bestFit="1" customWidth="1"/>
+    <col width="18.700000000000003" min="15" max="15" bestFit="1" customWidth="1"/>
+    <col width="18.700000000000003" min="16" max="16" bestFit="1" customWidth="1"/>
+    <col width="18.700000000000003" min="17" max="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -319,35 +361,50 @@
       </c>
       <c r="H1" s="0" t="inlineStr">
         <is>
+          <t>YYYY-Week</t>
+        </is>
+      </c>
+      <c r="I1" s="0" t="inlineStr">
+        <is>
+          <t>YYYY-MM</t>
+        </is>
+      </c>
+      <c r="J1" s="0" t="inlineStr">
+        <is>
+          <t>YYYY</t>
+        </is>
+      </c>
+      <c r="K1" s="0" t="inlineStr">
+        <is>
           <t>Cycle Time (days)</t>
         </is>
       </c>
-      <c r="I1" s="0" t="inlineStr">
+      <c r="L1" s="0" t="inlineStr">
         <is>
           <t>Current Age (days)</t>
         </is>
       </c>
-      <c r="J1" s="0" t="inlineStr">
+      <c r="M1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 1 day</t>
         </is>
       </c>
-      <c r="K1" s="0" t="inlineStr">
+      <c r="N1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 7 days</t>
         </is>
       </c>
-      <c r="L1" s="0" t="inlineStr">
+      <c r="O1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 14 days</t>
         </is>
       </c>
-      <c r="M1" s="0" t="inlineStr">
+      <c r="P1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 21 days</t>
         </is>
       </c>
-      <c r="N1" s="0" t="inlineStr">
+      <c r="Q1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 28 days</t>
         </is>
@@ -377,23 +434,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H2" s="0" t="n">
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t>2026-W10</t>
+        </is>
+      </c>
+      <c r="I2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J2" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K2" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="I2" s="0"/>
-      <c r="J2" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K2" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L2" s="0"/>
       <c r="M2" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -421,23 +491,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H3" s="0" t="n">
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>2026-W10</t>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J3" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K3" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="I3" s="0"/>
-      <c r="J3" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K3" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L3" s="0"/>
       <c r="M3" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N3" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -465,23 +548,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H4" s="0" t="n">
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t>2026-W11</t>
+        </is>
+      </c>
+      <c r="I4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J4" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K4" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K4" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L4" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L4" s="0"/>
       <c r="M4" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -509,23 +605,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H5" s="0" t="n">
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t>2026-W10</t>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J5" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K5" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K5" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L5" s="0"/>
       <c r="M5" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -553,23 +662,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H6" s="0" t="n">
+      <c r="H6" s="0" t="inlineStr">
+        <is>
+          <t>2026-W11</t>
+        </is>
+      </c>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J6" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K6" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L6" s="0"/>
       <c r="M6" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -597,23 +719,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H7" s="0" t="n">
+      <c r="H7" s="0" t="inlineStr">
+        <is>
+          <t>2026-W11</t>
+        </is>
+      </c>
+      <c r="I7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J7" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="I7" s="0"/>
-      <c r="J7" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K7" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L7" s="0"/>
       <c r="M7" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -641,23 +776,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H8" s="0" t="n">
+      <c r="H8" s="0" t="inlineStr">
+        <is>
+          <t>2026-W12</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J8" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="I8" s="0"/>
-      <c r="J8" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K8" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L8" s="0"/>
       <c r="M8" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -685,23 +833,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H9" s="0" t="n">
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t>2026-W12</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J9" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K9" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="I9" s="0"/>
-      <c r="J9" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K9" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L9" s="0"/>
       <c r="M9" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -729,23 +890,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H10" s="0" t="n">
+      <c r="H10" s="0" t="inlineStr">
+        <is>
+          <t>2026-W12</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J10" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K10" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="I10" s="0"/>
-      <c r="J10" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K10" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="L10" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L10" s="0"/>
       <c r="M10" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -773,23 +947,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H11" s="0" t="n">
+      <c r="H11" s="0" t="inlineStr">
+        <is>
+          <t>2026-W13</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J11" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K11" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="I11" s="0"/>
-      <c r="J11" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K11" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="L11" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L11" s="0"/>
       <c r="M11" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -817,23 +1004,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H12" s="0" t="n">
+      <c r="H12" s="0" t="inlineStr">
+        <is>
+          <t>2026-W13</t>
+        </is>
+      </c>
+      <c r="I12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="J12" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K12" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="I12" s="0"/>
-      <c r="J12" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K12" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="L12" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L12" s="0"/>
       <c r="M12" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -861,23 +1061,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H13" s="0" t="n">
+      <c r="H13" s="0" t="inlineStr">
+        <is>
+          <t>2026-W14</t>
+        </is>
+      </c>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="J13" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K13" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="I13" s="0"/>
-      <c r="J13" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K13" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="L13" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L13" s="0"/>
       <c r="M13" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="O13" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P13" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -905,23 +1118,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H14" s="0" t="n">
+      <c r="H14" s="0" t="inlineStr">
+        <is>
+          <t>2026-W14</t>
+        </is>
+      </c>
+      <c r="I14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="J14" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K14" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="I14" s="0"/>
-      <c r="J14" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K14" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="L14" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L14" s="0"/>
       <c r="M14" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="O14" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P14" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -949,23 +1175,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H15" s="0" t="n">
+      <c r="H15" s="0" t="inlineStr">
+        <is>
+          <t>2026-W14</t>
+        </is>
+      </c>
+      <c r="I15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="J15" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K15" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K15" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="L15" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L15" s="0"/>
       <c r="M15" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="O15" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P15" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -993,23 +1232,36 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="H16" s="0" t="n">
+      <c r="H16" s="0" t="inlineStr">
+        <is>
+          <t>2026-W15</t>
+        </is>
+      </c>
+      <c r="I16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="J16" s="0" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K16" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="I16" s="0"/>
-      <c r="J16" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="K16" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="L16" s="0" t="b">
-        <v>1</v>
-      </c>
+      <c r="L16" s="0"/>
       <c r="M16" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P16" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1036,14 +1288,17 @@
         </is>
       </c>
       <c r="H17" s="0"/>
-      <c r="I17" s="0" t="n">
-        <v>32</v>
-      </c>
+      <c r="I17" s="0"/>
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
-      <c r="L17" s="0"/>
+      <c r="L17" s="0" t="n">
+        <v>33</v>
+      </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
+      <c r="O17" s="0"/>
+      <c r="P17" s="0"/>
+      <c r="Q17" s="0"/>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -1068,14 +1323,17 @@
         </is>
       </c>
       <c r="H18" s="0"/>
-      <c r="I18" s="0" t="n">
-        <v>30</v>
-      </c>
+      <c r="I18" s="0"/>
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
-      <c r="L18" s="0"/>
+      <c r="L18" s="0" t="n">
+        <v>31</v>
+      </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
+      <c r="O18" s="0"/>
+      <c r="P18" s="0"/>
+      <c r="Q18" s="0"/>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -1100,14 +1358,17 @@
         </is>
       </c>
       <c r="H19" s="0"/>
-      <c r="I19" s="0" t="n">
-        <v>28</v>
-      </c>
+      <c r="I19" s="0"/>
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
-      <c r="L19" s="0"/>
+      <c r="L19" s="0" t="n">
+        <v>29</v>
+      </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>
+      <c r="O19" s="0"/>
+      <c r="P19" s="0"/>
+      <c r="Q19" s="0"/>
     </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="1"/>
@@ -1130,7 +1391,7 @@
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
   <headerFooter/>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId15"/>
 </worksheet>
 </file>
 
@@ -1146,7 +1407,7 @@
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
   <headerFooter/>
-  <drawing r:id="rId14"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
 
@@ -1162,7 +1423,7 @@
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
   <headerFooter/>
-  <drawing r:id="rId15"/>
+  <drawing r:id="rId17"/>
 </worksheet>
 </file>
 
@@ -1178,7 +1439,7 @@
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
   <headerFooter/>
-  <drawing r:id="rId16"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
 
@@ -1194,6 +1455,22 @@
   <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
   <headerFooter/>
-  <drawing r:id="rId17"/>
+  <drawing r:id="rId19"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
+  <sheetData/>
+  <sheetCalcPr fullCalcOnLoad="1"/>
+  <printOptions gridLines="0" headings="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1.0" bottom="1.0" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter/>
+  <drawing r:id="rId20"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: increase Aruba exit_timeout from 180 s to 600 s for CI reliability
The all_formats and extra_large_data Cucumber scenarios both invoke
`predictability-engine viz all_formats` which launches Chromium via
Playwright multiple times (pdf, a3_landscape, png, pptx).  On slow CI
machines running Alpine Linux with the system Chromium package the
combined render time exceeded the previous 180-second Aruba exit_timeout,
causing Aruba to kill the subprocess and report an empty exit status ("").

Raise the global timeout to 600 s (10 min) so all Playwright-heavy
scenarios have sufficient headroom on constrained CI hardware.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1292,7 +1292,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -1327,7 +1327,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -1362,7 +1362,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>

</xml_diff>

<commit_message>
fix: remove verify-fresh-install-windows step — no Windows runner or image exists
ruby:4.0.3-windowsservercore-ltsc2022 is not published to Docker Hub and
photocenter (the Windows agent) is offline. Woodpecker's failure: ignore does not
cover scheduling failures (no matching agent), so the step was blocking publish
from going green. Remove it until a working Windows runner and image are available.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1292,7 +1292,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -1327,7 +1327,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -1362,7 +1362,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>

</xml_diff>

<commit_message>
fix: move Windows verify step to dedicated pipeline targeting photocenter
platform: at step level is invalid in Woodpecker v3 (linter: "Additional
property platform is not allowed"). The step was being picked up by
photovault (Linux Docker) which tried to pull 'bat' as a Docker image,
causing failure despite failure: ignore.

Moved verify-fresh-install-windows into .woodpecker/verify-windows.yml
with platform: windows/amd64 at the pipeline level (valid) and
depends_on: [publish] so it waits for the gem to be pushed before
attempting to install it on photocenter (Windows, local backend).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1292,7 +1292,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -1327,7 +1327,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -1362,7 +1362,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>

</xml_diff>

<commit_message>
fix: bypass GCM on photocenter by overriding clone with token auth
Git Credential Manager (GCM) on Windows intercepts HTTPS git auth and
requires interactive OAuth which fails without a TTY. Disable the
credential helper and embed the Forgejo PAT directly in the clone URL
so the local-backend clone succeeds unattended.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1292,7 +1292,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -1327,7 +1327,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -1362,7 +1362,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>

</xml_diff>

<commit_message>
chore: bump version to 0.3.12
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1292,7 +1292,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -1327,7 +1327,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -1362,7 +1362,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>

</xml_diff>

<commit_message>
fix(ci): pin all Linux workflows to platform=linux agent label
The Windows Woodpecker exec-backend agent (photocenter) was accepting
pipeline jobs that had no labels, despite having WOODPECKER_FILTER_LABELS=
platform=windows configured. This caused publish, verify, jira-integration,
and predictability-engine workflows to land on the Windows exec agent,
where ruby:4.0.3-alpine Docker images cannot run, producing immediate
failures with no logs.

Add `labels: platform: linux` to every Linux workflow so Woodpecker
routes them exclusively to the Docker agent that advertises
WOODPECKER_AGENT_LABELS=platform=linux, making agent selection
deterministic regardless of the agent filter behaviour.

Also update Gemfile.lock to reflect the 0.3.15 version bump that was
missing from the previous chore commit.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1292,7 +1292,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -1327,7 +1327,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -1362,7 +1362,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>

</xml_diff>

<commit_message>
fix(gemspec): handle `.ruby-version` files with Ruby prefix
Update `required_ruby_version` parsing in the gemspec to handle `.ruby-version` files
containing a version prefixed with "ruby-", ensuring compatibility with updated `.ruby-version` format.
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1292,7 +1292,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -1327,7 +1327,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -1362,7 +1362,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>

</xml_diff>

<commit_message>
feat: add --url-prefix option to construct ticket URLs from item IDs
When CSV or Excel data lacks a url column, a prefix (e.g.
https://jira.example.com/browse/) can now be specified via:
  - CLI flag --url-prefix
  - CSV sidecar .yml: url_prefix: key
  - .predictability_engine.yml: top-level url_prefix: key (all sources)

CLI takes highest priority; sidecar overrides project config.
The file:// CSV fallback is skipped when a prefix is configured.

Also adds a URL column to CSV and XLSX raw data exports so ticket
links are included alongside the metrics data.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -301,7 +301,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="11.0" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -316,11 +316,12 @@
     <col width="7.700000000000001" min="10" max="10" bestFit="1" customWidth="1"/>
     <col width="22.0" min="11" max="11" bestFit="1" customWidth="1"/>
     <col width="23.1" min="12" max="12" bestFit="1" customWidth="1"/>
-    <col width="16.5" min="13" max="13" bestFit="1" customWidth="1"/>
-    <col width="17.6" min="14" max="14" bestFit="1" customWidth="1"/>
-    <col width="18.700000000000003" min="15" max="15" bestFit="1" customWidth="1"/>
+    <col width="92.4" min="13" max="13" bestFit="1" customWidth="1"/>
+    <col width="16.5" min="14" max="14" bestFit="1" customWidth="1"/>
+    <col width="17.6" min="15" max="15" bestFit="1" customWidth="1"/>
     <col width="18.700000000000003" min="16" max="16" bestFit="1" customWidth="1"/>
     <col width="18.700000000000003" min="17" max="17" bestFit="1" customWidth="1"/>
+    <col width="18.700000000000003" min="18" max="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -386,25 +387,30 @@
       </c>
       <c r="M1" s="0" t="inlineStr">
         <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="N1" s="0" t="inlineStr">
+        <is>
           <t>Done ≤ 1 day</t>
         </is>
       </c>
-      <c r="N1" s="0" t="inlineStr">
+      <c r="O1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 7 days</t>
         </is>
       </c>
-      <c r="O1" s="0" t="inlineStr">
+      <c r="P1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 14 days</t>
         </is>
       </c>
-      <c r="P1" s="0" t="inlineStr">
+      <c r="Q1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 21 days</t>
         </is>
       </c>
-      <c r="Q1" s="0" t="inlineStr">
+      <c r="R1" s="0" t="inlineStr">
         <is>
           <t>Done ≤ 28 days</t>
         </is>
@@ -451,11 +457,13 @@
         <v>5</v>
       </c>
       <c r="L2" s="0"/>
-      <c r="M2" s="0" t="b">
-        <v>0</v>
+      <c r="M2" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N2" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" s="0" t="b">
         <v>1</v>
@@ -464,6 +472,9 @@
         <v>1</v>
       </c>
       <c r="Q2" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R2" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -508,11 +519,13 @@
         <v>3</v>
       </c>
       <c r="L3" s="0"/>
-      <c r="M3" s="0" t="b">
-        <v>0</v>
+      <c r="M3" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N3" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" s="0" t="b">
         <v>1</v>
@@ -521,6 +534,9 @@
         <v>1</v>
       </c>
       <c r="Q3" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R3" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -565,11 +581,13 @@
         <v>6</v>
       </c>
       <c r="L4" s="0"/>
-      <c r="M4" s="0" t="b">
-        <v>0</v>
+      <c r="M4" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N4" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" s="0" t="b">
         <v>1</v>
@@ -578,6 +596,9 @@
         <v>1</v>
       </c>
       <c r="Q4" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R4" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -622,11 +643,13 @@
         <v>2</v>
       </c>
       <c r="L5" s="0"/>
-      <c r="M5" s="0" t="b">
-        <v>0</v>
+      <c r="M5" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N5" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" s="0" t="b">
         <v>1</v>
@@ -635,6 +658,9 @@
         <v>1</v>
       </c>
       <c r="Q5" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R5" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -679,11 +705,13 @@
         <v>5</v>
       </c>
       <c r="L6" s="0"/>
-      <c r="M6" s="0" t="b">
-        <v>0</v>
+      <c r="M6" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N6" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" s="0" t="b">
         <v>1</v>
@@ -692,6 +720,9 @@
         <v>1</v>
       </c>
       <c r="Q6" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R6" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -736,11 +767,13 @@
         <v>6</v>
       </c>
       <c r="L7" s="0"/>
-      <c r="M7" s="0" t="b">
-        <v>0</v>
+      <c r="M7" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N7" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="0" t="b">
         <v>1</v>
@@ -749,6 +782,9 @@
         <v>1</v>
       </c>
       <c r="Q7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R7" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -793,11 +829,13 @@
         <v>7</v>
       </c>
       <c r="L8" s="0"/>
-      <c r="M8" s="0" t="b">
-        <v>0</v>
+      <c r="M8" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N8" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="0" t="b">
         <v>1</v>
@@ -806,6 +844,9 @@
         <v>1</v>
       </c>
       <c r="Q8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R8" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -850,11 +891,13 @@
         <v>7</v>
       </c>
       <c r="L9" s="0"/>
-      <c r="M9" s="0" t="b">
-        <v>0</v>
+      <c r="M9" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N9" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" s="0" t="b">
         <v>1</v>
@@ -863,6 +906,9 @@
         <v>1</v>
       </c>
       <c r="Q9" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R9" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -907,11 +953,13 @@
         <v>7</v>
       </c>
       <c r="L10" s="0"/>
-      <c r="M10" s="0" t="b">
-        <v>0</v>
+      <c r="M10" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N10" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O10" s="0" t="b">
         <v>1</v>
@@ -920,6 +968,9 @@
         <v>1</v>
       </c>
       <c r="Q10" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R10" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -964,19 +1015,24 @@
         <v>8</v>
       </c>
       <c r="L11" s="0"/>
-      <c r="M11" s="0" t="b">
-        <v>0</v>
+      <c r="M11" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N11" s="0" t="b">
         <v>0</v>
       </c>
       <c r="O11" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P11" s="0" t="b">
         <v>1</v>
       </c>
       <c r="Q11" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R11" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1021,19 +1077,24 @@
         <v>9</v>
       </c>
       <c r="L12" s="0"/>
-      <c r="M12" s="0" t="b">
-        <v>0</v>
+      <c r="M12" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N12" s="0" t="b">
         <v>0</v>
       </c>
       <c r="O12" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12" s="0" t="b">
         <v>1</v>
       </c>
       <c r="Q12" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R12" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1078,19 +1139,24 @@
         <v>11</v>
       </c>
       <c r="L13" s="0"/>
-      <c r="M13" s="0" t="b">
-        <v>0</v>
+      <c r="M13" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N13" s="0" t="b">
         <v>0</v>
       </c>
       <c r="O13" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P13" s="0" t="b">
         <v>1</v>
       </c>
       <c r="Q13" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R13" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1135,19 +1201,24 @@
         <v>11</v>
       </c>
       <c r="L14" s="0"/>
-      <c r="M14" s="0" t="b">
-        <v>0</v>
+      <c r="M14" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N14" s="0" t="b">
         <v>0</v>
       </c>
       <c r="O14" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P14" s="0" t="b">
         <v>1</v>
       </c>
       <c r="Q14" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R14" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1192,19 +1263,24 @@
         <v>11</v>
       </c>
       <c r="L15" s="0"/>
-      <c r="M15" s="0" t="b">
-        <v>0</v>
+      <c r="M15" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N15" s="0" t="b">
         <v>0</v>
       </c>
       <c r="O15" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P15" s="0" t="b">
         <v>1</v>
       </c>
       <c r="Q15" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R15" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1249,19 +1325,24 @@
         <v>12</v>
       </c>
       <c r="L16" s="0"/>
-      <c r="M16" s="0" t="b">
-        <v>0</v>
+      <c r="M16" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
       </c>
       <c r="N16" s="0" t="b">
         <v>0</v>
       </c>
       <c r="O16" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P16" s="0" t="b">
         <v>1</v>
       </c>
       <c r="Q16" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="R16" s="0" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1294,11 +1375,16 @@
       <c r="L17" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="M17" s="0"/>
+      <c r="M17" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
+      </c>
       <c r="N17" s="0"/>
       <c r="O17" s="0"/>
       <c r="P17" s="0"/>
       <c r="Q17" s="0"/>
+      <c r="R17" s="0"/>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -1329,11 +1415,16 @@
       <c r="L18" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="M18" s="0"/>
+      <c r="M18" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
+      </c>
       <c r="N18" s="0"/>
       <c r="O18" s="0"/>
       <c r="P18" s="0"/>
       <c r="Q18" s="0"/>
+      <c r="R18" s="0"/>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -1364,11 +1455,16 @@
       <c r="L19" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="M19" s="0"/>
+      <c r="M19" s="0" t="inlineStr">
+        <is>
+          <t>file:///home/cbroult/work/ruby/predictability-engine/data/samples/sample_data.csv</t>
+        </is>
+      </c>
       <c r="N19" s="0"/>
       <c r="O19" s="0"/>
       <c r="P19" s="0"/>
       <c r="Q19" s="0"/>
+      <c r="R19" s="0"/>
     </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix(viz): reduce FCFD right padding and add top padding for confidence labels
Vertical confidence rule labels (rotated -45°) had ~43px of excess white
space on the right side because the 110px right padding exceeded label needs.
The top had no padding, clipping the label tips above the plateau line.

New padding { right: 80, top: 30 } aligns the reserved space with actual
label geometry: the scale's natural nice-mode extension (~31px) provides the
remaining buffer between the rightmost rule and the padding zone boundary.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(ci): replace UTF-8 em-dashes with ASCII hyphens in PowerShell scripts
Windows PowerShell 5.x reads PS1 files without BOM using the system code
page (cp1252). The UTF-8 em-dash bytes (E2 80 94) decode as a right double
quotation mark (U+201D, cp1252 byte 0x94), which PowerShell treats as a
string terminator. This caused a spurious parse error on the else-block
brace in verify-fresh-install-windows.ps1, making the verify-windows CI
step fail immediately with "Missing closing '}'".

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(publish): wire OTP seed env var and fix bundle install in publish-rubygems step
Three bugs prevented rubygems.org publishing:
1. Repos.rubygems_otp_seed_env_var was nil (default), so gem push was called
   without --otp even though RUBYGEMS_OTP_SEED was set — MFA-enabled accounts
   rejected every push silently.
2. The publish-rubygems CI step had no JIRA_ENV, so bundle install tried to
   reach gems.cbp-org.internal (internal source in Gemfile) but had no
   extra_hosts or CA cert — the step failed before rake ever ran.
3. GemPublisher#publish never raises on failure; added a successful_repos
   check so the step actually fails the pipeline when publishing fails.

Extracted RubygemsPublisher class to rakelib/ so the logic is testable; spec
covers config wiring, no-gem-file guard, failure raise, and success path.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(ci): run @npm_required scenarios in verify; promote Playwright env vars to block
- Add `features_npm` to the `verify` task so @npm_required Cucumber
  scenarios (Playwright install/update checks) run as part of CI.
- Move PLAYWRIGHT_SKIP_BROWSER_DOWNLOAD and PLAYWRIGHT_CHROMIUM_EXECUTABLE_PATH
  from inline command prefixes to the step environment block so they apply
  to all commands including `rake verify`.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(todo): update Multi-OS section to reflect completed CI work
Linux and Docker are fully covered. Windows runs as best-effort.
Mac has no agent but the code is platform-neutral.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(deps): upgrade rake-gem-maintenance to 0.2.2
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ci(windows): install from rubygems.org and depend on verify instead of publish
The Windows CI step was blocked indefinitely because it depended on the
publish workflow, which requires Docker networking that keeps timing out
on the CI server. End users install from rubygems.org anyway, so switch
to that source and make verify-windows depend on verify instead.

Also removes the CBP_ORG_CA_CERT block — no longer needed since we are
not connecting to the internal gem registry.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(ci): artifact-first publish — gem stored on nexus raw before any registry push
Build X.Y.Z gem in publish.yml, upload to nexus raw artifact store.
verify-linux and verify-windows download and install --local; only
promote.yml touches the gem registry after both platforms pass.
Also switches GitHub push from HTTPS PAT to SSH deploy key.
Extracted hook shared boilerplate to .claude/hooks/hook-lib.sh (jscpd DRY).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(ci): avoid update-ca-certificates in verify-linux; use env-based cert trust
update-ca-certificates fails on this runner with "Device or resource busy"
because Docker bind-mounts /etc/ssl/certs/ca-certificates.crt from the host,
making the atomic mv(1) inside the tool fail at a EXDEV/EBUSY boundary.

Instead: decode the CA cert to /tmp/cbp-ca.crt, build a merged bundle at
/tmp/ca-bundle.crt (system CAs + custom CA), then export SSL_CERT_FILE and
NODE_EXTRA_CA_CERTS so Ruby and Node respect the bundle without touching
any system-owned paths.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(jscpd): remove redundant \$LOAD_PATH from jira-project-setup script
jira_project_setup.rb uses require_relative for all PE lib files, so the
\$LOAD_PATH.unshift in the wrapper script was unused and caused a jscpd
clone match with the identical block in bin/predictability-engine.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data/dashboard.xlsx
+++ b/data/samples/reports/sample_data/dashboard.xlsx
@@ -1373,7 +1373,7 @@
       <c r="J17" s="0"/>
       <c r="K17" s="0"/>
       <c r="L17" s="0" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M17" s="0" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
       <c r="J18" s="0"/>
       <c r="K18" s="0"/>
       <c r="L18" s="0" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M18" s="0" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
       <c r="J19" s="0"/>
       <c r="K19" s="0"/>
       <c r="L19" s="0" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M19" s="0" t="inlineStr">
         <is>

</xml_diff>